<commit_message>
updated admin dashboard for bypass the orders
</commit_message>
<xml_diff>
--- a/sample-orders.xlsx
+++ b/sample-orders.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -444,16 +444,93 @@
         <v>9876543212</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>ORD-1004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Neha Gupta</v>
+      </c>
+      <c r="C5" t="str">
+        <v>9876543213</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>ORD-1005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Isha Kapoor</v>
+      </c>
+      <c r="C6" t="str">
+        <v>9876543214</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>ORD-1006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Kabir Singh</v>
+      </c>
+      <c r="C7" t="str">
+        <v>9876543215</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>ORD-1007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Maya Patel</v>
+      </c>
+      <c r="C8" t="str">
+        <v>9876543216</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>ORD-1008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Aditya Rao</v>
+      </c>
+      <c r="C9" t="str">
+        <v>9876543217</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>ORD-1009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Sara Khan</v>
+      </c>
+      <c r="C10" t="str">
+        <v>9876543218</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>ORD-1010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Vikram Joshi</v>
+      </c>
+      <c r="C11" t="str">
+        <v>9876543219</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C11"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -557,9 +634,264 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>ORD-1003</v>
+      </c>
+      <c r="B7" t="str">
+        <v>USB-C Cable</v>
+      </c>
+      <c r="C7" t="str">
+        <v>SKU-006</v>
+      </c>
+      <c r="D7" t="str">
+        <v>1m braided charging cable</v>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>ORD-1004</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Smart Watch</v>
+      </c>
+      <c r="C8" t="str">
+        <v>SKU-007</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Fitness smart watch</v>
+      </c>
+      <c r="E8" t="str">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>ORD-1004</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Watch Strap</v>
+      </c>
+      <c r="C9" t="str">
+        <v>SKU-008</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Silicone replacement strap</v>
+      </c>
+      <c r="E9" t="str">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>ORD-1005</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Laptop Stand</v>
+      </c>
+      <c r="C10" t="str">
+        <v>SKU-009</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Adjustable aluminum stand</v>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>ORD-1005</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Desk Lamp</v>
+      </c>
+      <c r="C11" t="str">
+        <v>SKU-010</v>
+      </c>
+      <c r="D11" t="str">
+        <v>LED desk lamp warm white</v>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>ORD-1006</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Bluetooth Speaker</v>
+      </c>
+      <c r="C12" t="str">
+        <v>SKU-011</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Portable speaker 20W</v>
+      </c>
+      <c r="E12" t="str">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>ORD-1006</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Travel Pouch</v>
+      </c>
+      <c r="C13" t="str">
+        <v>SKU-012</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Carry pouch for accessories</v>
+      </c>
+      <c r="E13" t="str">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>ORD-1007</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Phone Case</v>
+      </c>
+      <c r="C14" t="str">
+        <v>SKU-013</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Shockproof case for phone</v>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>ORD-1007</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Screen Protector</v>
+      </c>
+      <c r="C15" t="str">
+        <v>SKU-014</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Tempered glass protector</v>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>ORD-1008</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Tablet Cover</v>
+      </c>
+      <c r="C16" t="str">
+        <v>SKU-015</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Magnetic folio cover</v>
+      </c>
+      <c r="E16" t="str">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>ORD-1008</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Stylus Pen</v>
+      </c>
+      <c r="C17" t="str">
+        <v>SKU-016</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Active stylus pen</v>
+      </c>
+      <c r="E17" t="str">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>ORD-1009</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Gaming Mouse</v>
+      </c>
+      <c r="C18" t="str">
+        <v>SKU-017</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Wireless gaming mouse</v>
+      </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>ORD-1009</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Mouse Pad</v>
+      </c>
+      <c r="C19" t="str">
+        <v>SKU-018</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Large stitched mouse pad</v>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>ORD-1010</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Backpack</v>
+      </c>
+      <c r="C20" t="str">
+        <v>SKU-019</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Water resistant backpack</v>
+      </c>
+      <c r="E20" t="str">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>ORD-1010</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Notebook Set</v>
+      </c>
+      <c r="C21" t="str">
+        <v>SKU-020</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Set of 3 ruled notebooks</v>
+      </c>
+      <c r="E21" t="str">
+        <v>40</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>